<commit_message>
dumping the current state of the code here
</commit_message>
<xml_diff>
--- a/gas_net/data/data_files/Gaslib_40/networkData.xlsx
+++ b/gas_net/data/data_files/Gaslib_40/networkData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ssnaik\Biegler\gas_networks_italy\gas_networks\gas_net\data\data_files\Gaslib_40\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4B148A5-1554-4CDF-8470-8729C0B6EFC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D865C29D-1C06-4F08-883B-9779052C0876}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,20 @@
     <sheet name="Stations" sheetId="3" r:id="rId3"/>
     <sheet name="Arcs" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -707,9 +720,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G41"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -730,7 +743,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -750,7 +763,7 @@
         <v>7.1514568006000001</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -770,7 +783,7 @@
         <v>6.40592572072</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -790,7 +803,7 @@
         <v>8.4621655320400002</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -810,7 +823,7 @@
         <v>6.9854010493200001</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -830,7 +843,7 @@
         <v>7.4443755311900004</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -850,7 +863,7 @@
         <v>6.73248116159</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -870,7 +883,7 @@
         <v>8.9411702828399999</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -890,7 +903,7 @@
         <v>8.5833395540000001</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -910,7 +923,7 @@
         <v>7.3753776974200003</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -930,7 +943,7 @@
         <v>7.1753586073599998</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -950,7 +963,7 @@
         <v>6.7041298791399999</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -970,7 +983,7 @@
         <v>7.3914117238100001</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -990,7 +1003,7 @@
         <v>8.42123710095</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -1010,7 +1023,7 @@
         <v>7.0605075488400004</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>20</v>
       </c>
@@ -1030,7 +1043,7 @@
         <v>7.4457078406599999</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -1050,7 +1063,7 @@
         <v>6.68272868748</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -1070,7 +1083,7 @@
         <v>8.90117691783</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -1090,7 +1103,7 @@
         <v>6.9707746782799997</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -1110,7 +1123,7 @@
         <v>6.8901153727300004</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>25</v>
       </c>
@@ -1130,7 +1143,7 @@
         <v>7.1600196325600001</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>26</v>
       </c>
@@ -1150,7 +1163,7 @@
         <v>8.5229746891700007</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>27</v>
       </c>
@@ -1170,7 +1183,7 @@
         <v>9.4346584907499995</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>28</v>
       </c>
@@ -1190,7 +1203,7 @@
         <v>7.53102691462</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>29</v>
       </c>
@@ -1213,7 +1226,7 @@
         <v>6.0379656315299997</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>30</v>
       </c>
@@ -1236,7 +1249,7 @@
         <v>8.9727930560200004</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>31</v>
       </c>
@@ -1259,7 +1272,7 @@
         <v>6.8375660756499999</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>32</v>
       </c>
@@ -1279,7 +1292,7 @@
         <v>7.2972825175800002</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>33</v>
       </c>
@@ -1299,7 +1312,7 @@
         <v>6.0766343127700004</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>34</v>
       </c>
@@ -1319,7 +1332,7 @@
         <v>7.0121622871099998</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>35</v>
       </c>
@@ -1339,7 +1352,7 @@
         <v>6.9910068056399997</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>36</v>
       </c>
@@ -1359,7 +1372,7 @@
         <v>7.3343218248599999</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>37</v>
       </c>
@@ -1379,7 +1392,7 @@
         <v>7.1259504410399996</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>38</v>
       </c>
@@ -1399,7 +1412,7 @@
         <v>7.2293030868199999</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>39</v>
       </c>
@@ -1419,7 +1432,7 @@
         <v>8.2267773593700007</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>40</v>
       </c>
@@ -1439,7 +1452,7 @@
         <v>8.5682177229499992</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>41</v>
       </c>
@@ -1459,7 +1472,7 @@
         <v>6.6172322377899997</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>42</v>
       </c>
@@ -1479,7 +1492,7 @@
         <v>6.5567145582800004</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>43</v>
       </c>
@@ -1499,7 +1512,7 @@
         <v>6.6466959069599998</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>44</v>
       </c>
@@ -1519,7 +1532,7 @@
         <v>6.4827114548100004</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>45</v>
       </c>
@@ -1547,9 +1560,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K40"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>46</v>
@@ -1582,7 +1595,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>56</v>
       </c>
@@ -1590,13 +1603,14 @@
         <v>65057.174267899987</v>
       </c>
       <c r="C2">
-        <v>0.50265482457436694</v>
+        <f xml:space="preserve"> 3.141*E2^2/4</f>
+        <v>0.78525</v>
       </c>
       <c r="D2">
         <v>2.513274122871834</v>
       </c>
       <c r="E2">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F2">
         <v>5.0000000000000002E-5</v>
@@ -1617,7 +1631,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>57</v>
       </c>
@@ -1625,13 +1639,14 @@
         <v>32449.372045299999</v>
       </c>
       <c r="C3">
-        <v>0.78539816339744828</v>
+        <f t="shared" ref="C3:C40" si="0" xml:space="preserve"> 3.141*E3^2/4</f>
+        <v>3.141</v>
       </c>
       <c r="D3">
         <v>3.1415926535897931</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3">
         <v>5.0000000000000002E-5</v>
@@ -1652,7 +1667,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>58</v>
       </c>
@@ -1660,13 +1675,14 @@
         <v>13071.0852297</v>
       </c>
       <c r="C4">
-        <v>0.78539816339744828</v>
+        <f t="shared" si="0"/>
+        <v>3.141</v>
       </c>
       <c r="D4">
         <v>3.1415926535897931</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4">
         <v>5.0000000000000002E-5</v>
@@ -1687,7 +1703,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>59</v>
       </c>
@@ -1695,13 +1711,14 @@
         <v>12766.7034136</v>
       </c>
       <c r="C5">
-        <v>0.78539816339744828</v>
+        <f t="shared" si="0"/>
+        <v>3.141</v>
       </c>
       <c r="D5">
         <v>3.1415926535897931</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F5">
         <v>5.0000000000000002E-5</v>
@@ -1722,7 +1739,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>60</v>
       </c>
@@ -1730,13 +1747,14 @@
         <v>76893.550756800003</v>
       </c>
       <c r="C6">
-        <v>0.50265482457436694</v>
+        <f t="shared" si="0"/>
+        <v>0.78525</v>
       </c>
       <c r="D6">
         <v>2.513274122871834</v>
       </c>
       <c r="E6">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F6">
         <v>5.0000000000000002E-5</v>
@@ -1757,7 +1775,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>61</v>
       </c>
@@ -1765,13 +1783,14 @@
         <v>36061.009874700001</v>
       </c>
       <c r="C7">
-        <v>0.50265482457436694</v>
+        <f t="shared" si="0"/>
+        <v>0.78525</v>
       </c>
       <c r="D7">
         <v>2.513274122871834</v>
       </c>
       <c r="E7">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F7">
         <v>5.0000000000000002E-5</v>
@@ -1792,7 +1811,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>62</v>
       </c>
@@ -1800,13 +1819,14 @@
         <v>47488.283852300003</v>
       </c>
       <c r="C8">
-        <v>0.50265482457436694</v>
+        <f t="shared" si="0"/>
+        <v>0.78525</v>
       </c>
       <c r="D8">
         <v>2.513274122871834</v>
       </c>
       <c r="E8">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F8">
         <v>5.0000000000000002E-5</v>
@@ -1827,7 +1847,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>63</v>
       </c>
@@ -1835,7 +1855,8 @@
         <v>20322.2054259</v>
       </c>
       <c r="C9">
-        <v>0.28274333882308139</v>
+        <f t="shared" si="0"/>
+        <v>0.28269</v>
       </c>
       <c r="D9">
         <v>1.8849555921538761</v>
@@ -1862,7 +1883,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>64</v>
       </c>
@@ -1870,13 +1891,14 @@
         <v>32921.259814999998</v>
       </c>
       <c r="C10">
-        <v>0.50265482457436694</v>
+        <f t="shared" si="0"/>
+        <v>0.78525</v>
       </c>
       <c r="D10">
         <v>2.513274122871834</v>
       </c>
       <c r="E10">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F10">
         <v>5.0000000000000002E-5</v>
@@ -1897,7 +1919,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>65</v>
       </c>
@@ -1905,13 +1927,14 @@
         <v>39036.041811399999</v>
       </c>
       <c r="C11">
-        <v>0.50265482457436694</v>
+        <f t="shared" si="0"/>
+        <v>0.78525</v>
       </c>
       <c r="D11">
         <v>2.513274122871834</v>
       </c>
       <c r="E11">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F11">
         <v>5.0000000000000002E-5</v>
@@ -1932,7 +1955,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>66</v>
       </c>
@@ -1940,13 +1963,14 @@
         <v>21557.5661917</v>
       </c>
       <c r="C12">
-        <v>0.78539816339744828</v>
+        <f t="shared" si="0"/>
+        <v>3.141</v>
       </c>
       <c r="D12">
         <v>3.1415926535897931</v>
       </c>
       <c r="E12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F12">
         <v>5.0000000000000002E-5</v>
@@ -1967,7 +1991,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>67</v>
       </c>
@@ -1975,13 +1999,14 @@
         <v>31179.6191038</v>
       </c>
       <c r="C13">
-        <v>0.50265482457436694</v>
+        <f t="shared" si="0"/>
+        <v>0.78525</v>
       </c>
       <c r="D13">
         <v>2.513274122871834</v>
       </c>
       <c r="E13">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F13">
         <v>5.0000000000000002E-5</v>
@@ -2002,7 +2027,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>68</v>
       </c>
@@ -2010,7 +2035,8 @@
         <v>14043.1135378</v>
       </c>
       <c r="C14">
-        <v>0.12566370614359171</v>
+        <f t="shared" si="0"/>
+        <v>0.12564000000000003</v>
       </c>
       <c r="D14">
         <v>1.256637061435917</v>
@@ -2037,7 +2063,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>69</v>
       </c>
@@ -2045,13 +2071,14 @@
         <v>58218.969553100003</v>
       </c>
       <c r="C15">
-        <v>0.50265482457436694</v>
+        <f t="shared" si="0"/>
+        <v>0.78525</v>
       </c>
       <c r="D15">
         <v>2.513274122871834</v>
       </c>
       <c r="E15">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F15">
         <v>5.0000000000000002E-5</v>
@@ -2072,7 +2099,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>70</v>
       </c>
@@ -2080,7 +2107,8 @@
         <v>20634.698268799999</v>
       </c>
       <c r="C16">
-        <v>0.28274333882308139</v>
+        <f t="shared" si="0"/>
+        <v>0.28269</v>
       </c>
       <c r="D16">
         <v>1.8849555921538761</v>
@@ -2107,7 +2135,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>71</v>
       </c>
@@ -2115,13 +2143,14 @@
         <v>3479.4546655200002</v>
       </c>
       <c r="C17">
-        <v>0.50265482457436694</v>
+        <f t="shared" si="0"/>
+        <v>0.78525</v>
       </c>
       <c r="D17">
         <v>2.513274122871834</v>
       </c>
       <c r="E17">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F17">
         <v>1.2E-5</v>
@@ -2142,7 +2171,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>72</v>
       </c>
@@ -2150,7 +2179,8 @@
         <v>3802.5866770500002</v>
       </c>
       <c r="C18">
-        <v>0.28274333882308139</v>
+        <f t="shared" si="0"/>
+        <v>0.28269</v>
       </c>
       <c r="D18">
         <v>1.8849555921538761</v>
@@ -2177,7 +2207,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>73</v>
       </c>
@@ -2185,13 +2215,14 @@
         <v>18136.597291800001</v>
       </c>
       <c r="C19">
-        <v>0.78539816339744828</v>
+        <f t="shared" si="0"/>
+        <v>3.141</v>
       </c>
       <c r="D19">
         <v>3.1415926535897931</v>
       </c>
       <c r="E19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F19">
         <v>5.0000000000000002E-5</v>
@@ -2212,7 +2243,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>74</v>
       </c>
@@ -2220,7 +2251,8 @@
         <v>10452.031177999999</v>
       </c>
       <c r="C20">
-        <v>0.28274333882308139</v>
+        <f t="shared" si="0"/>
+        <v>0.28269</v>
       </c>
       <c r="D20">
         <v>1.8849555921538761</v>
@@ -2247,7 +2279,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>75</v>
       </c>
@@ -2255,7 +2287,8 @@
         <v>65532.212711200002</v>
       </c>
       <c r="C21">
-        <v>0.50265482457436694</v>
+        <f t="shared" si="0"/>
+        <v>0.50256000000000012</v>
       </c>
       <c r="D21">
         <v>2.513274122871834</v>
@@ -2282,7 +2315,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>76</v>
       </c>
@@ -2290,13 +2323,14 @@
         <v>3418.0082512499998</v>
       </c>
       <c r="C22">
-        <v>0.78539816339744828</v>
+        <f t="shared" si="0"/>
+        <v>3.141</v>
       </c>
       <c r="D22">
         <v>3.1415926535897931</v>
       </c>
       <c r="E22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F22">
         <v>1.2E-5</v>
@@ -2317,7 +2351,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>77</v>
       </c>
@@ -2325,13 +2359,14 @@
         <v>12397.3521636</v>
       </c>
       <c r="C23">
-        <v>0.50265482457436694</v>
+        <f t="shared" si="0"/>
+        <v>0.78525</v>
       </c>
       <c r="D23">
         <v>2.513274122871834</v>
       </c>
       <c r="E23">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F23">
         <v>5.0000000000000002E-5</v>
@@ -2352,7 +2387,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>78</v>
       </c>
@@ -2360,7 +2395,8 @@
         <v>10586.1294733</v>
       </c>
       <c r="C24">
-        <v>0.28274333882308139</v>
+        <f t="shared" si="0"/>
+        <v>0.28269</v>
       </c>
       <c r="D24">
         <v>1.8849555921538761</v>
@@ -2387,7 +2423,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>79</v>
       </c>
@@ -2395,7 +2431,8 @@
         <v>35218.839086699998</v>
       </c>
       <c r="C25">
-        <v>0.28274333882308139</v>
+        <f t="shared" si="0"/>
+        <v>0.28269</v>
       </c>
       <c r="D25">
         <v>1.8849555921538761</v>
@@ -2422,7 +2459,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>80</v>
       </c>
@@ -2430,13 +2467,14 @@
         <v>22224.1532472</v>
       </c>
       <c r="C26">
-        <v>0.50265482457436694</v>
+        <f t="shared" si="0"/>
+        <v>0.78525</v>
       </c>
       <c r="D26">
         <v>2.513274122871834</v>
       </c>
       <c r="E26">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F26">
         <v>5.0000000000000002E-5</v>
@@ -2457,7 +2495,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>81</v>
       </c>
@@ -2465,7 +2503,8 @@
         <v>10022.7829812</v>
       </c>
       <c r="C27">
-        <v>0.28274333882308139</v>
+        <f t="shared" si="0"/>
+        <v>0.28269</v>
       </c>
       <c r="D27">
         <v>1.8849555921538761</v>
@@ -2492,7 +2531,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>82</v>
       </c>
@@ -2500,7 +2539,8 @@
         <v>38659.824363</v>
       </c>
       <c r="C28">
-        <v>0.12566370614359171</v>
+        <f t="shared" si="0"/>
+        <v>0.12564000000000003</v>
       </c>
       <c r="D28">
         <v>1.256637061435917</v>
@@ -2527,7 +2567,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>83</v>
       </c>
@@ -2535,13 +2575,14 @@
         <v>6998.0537787200001</v>
       </c>
       <c r="C29">
-        <v>0.78539816339744828</v>
+        <f t="shared" si="0"/>
+        <v>3.141</v>
       </c>
       <c r="D29">
         <v>3.1415926535897931</v>
       </c>
       <c r="E29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F29">
         <v>5.0000000000000002E-5</v>
@@ -2562,7 +2603,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>84</v>
       </c>
@@ -2570,7 +2611,8 @@
         <v>18017.8496012</v>
       </c>
       <c r="C30">
-        <v>0.28274333882308139</v>
+        <f t="shared" si="0"/>
+        <v>0.28269</v>
       </c>
       <c r="D30">
         <v>1.8849555921538761</v>
@@ -2597,7 +2639,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>85</v>
       </c>
@@ -2605,13 +2647,14 @@
         <v>86690.265566799993</v>
       </c>
       <c r="C31">
-        <v>0.50265482457436694</v>
+        <f t="shared" si="0"/>
+        <v>0.78525</v>
       </c>
       <c r="D31">
         <v>2.513274122871834</v>
       </c>
       <c r="E31">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F31">
         <v>5.0000000000000002E-5</v>
@@ -2632,7 +2675,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>86</v>
       </c>
@@ -2640,13 +2683,14 @@
         <v>49866.148387499998</v>
       </c>
       <c r="C32">
-        <v>0.50265482457436694</v>
+        <f t="shared" si="0"/>
+        <v>0.78525</v>
       </c>
       <c r="D32">
         <v>2.513274122871834</v>
       </c>
       <c r="E32">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F32">
         <v>5.0000000000000002E-5</v>
@@ -2667,7 +2711,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>87</v>
       </c>
@@ -2675,7 +2719,8 @@
         <v>19303.192019599999</v>
       </c>
       <c r="C33">
-        <v>0.28274333882308139</v>
+        <f t="shared" si="0"/>
+        <v>0.28269</v>
       </c>
       <c r="D33">
         <v>1.8849555921538761</v>
@@ -2702,7 +2747,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>88</v>
       </c>
@@ -2710,7 +2755,8 @@
         <v>12015.8748344</v>
       </c>
       <c r="C34">
-        <v>0.12566370614359171</v>
+        <f t="shared" si="0"/>
+        <v>0.12564000000000003</v>
       </c>
       <c r="D34">
         <v>1.256637061435917</v>
@@ -2737,7 +2783,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>89</v>
       </c>
@@ -2745,13 +2791,14 @@
         <v>18969.412711100002</v>
       </c>
       <c r="C35">
-        <v>0.78539816339744828</v>
+        <f t="shared" si="0"/>
+        <v>3.141</v>
       </c>
       <c r="D35">
         <v>3.1415926535897931</v>
       </c>
       <c r="E35">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F35">
         <v>5.0000000000000002E-5</v>
@@ -2772,7 +2819,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>90</v>
       </c>
@@ -2780,7 +2827,8 @@
         <v>16579.3259985</v>
       </c>
       <c r="C36">
-        <v>0.28274333882308139</v>
+        <f t="shared" si="0"/>
+        <v>0.28269</v>
       </c>
       <c r="D36">
         <v>1.8849555921538761</v>
@@ -2807,7 +2855,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>91</v>
       </c>
@@ -2815,7 +2863,8 @@
         <v>3067.54743994</v>
       </c>
       <c r="C37">
-        <v>0.28274333882308139</v>
+        <f t="shared" si="0"/>
+        <v>0.28269</v>
       </c>
       <c r="D37">
         <v>1.8849555921538761</v>
@@ -2842,7 +2891,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>92</v>
       </c>
@@ -2850,7 +2899,8 @@
         <v>66036.594630899999</v>
       </c>
       <c r="C38">
-        <v>0.28274333882308139</v>
+        <f t="shared" si="0"/>
+        <v>0.28269</v>
       </c>
       <c r="D38">
         <v>1.8849555921538761</v>
@@ -2877,7 +2927,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>93</v>
       </c>
@@ -2885,13 +2935,14 @@
         <v>26427.481645299998</v>
       </c>
       <c r="C39">
-        <v>0.50265482457436694</v>
+        <f t="shared" si="0"/>
+        <v>0.78525</v>
       </c>
       <c r="D39">
         <v>2.513274122871834</v>
       </c>
       <c r="E39">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F39">
         <v>5.0000000000000002E-5</v>
@@ -2912,7 +2963,7 @@
         <v>0.86</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>94</v>
       </c>
@@ -2920,13 +2971,14 @@
         <v>32868.2025259</v>
       </c>
       <c r="C40">
-        <v>0.50265482457436694</v>
+        <f t="shared" si="0"/>
+        <v>0.78525</v>
       </c>
       <c r="D40">
         <v>2.513274122871834</v>
       </c>
       <c r="E40">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F40">
         <v>5.0000000000000002E-5</v>
@@ -2955,9 +3007,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>95</v>
@@ -2972,7 +3024,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>99</v>
       </c>
@@ -2986,7 +3038,7 @@
         <v>2424387224.3367658</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>100</v>
       </c>
@@ -3000,7 +3052,7 @@
         <v>2424387224.3367658</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>101</v>
       </c>
@@ -3014,7 +3066,7 @@
         <v>2424387224.3367658</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>102</v>
       </c>
@@ -3028,7 +3080,7 @@
         <v>2424387224.3367658</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>103</v>
       </c>
@@ -3042,7 +3094,7 @@
         <v>2424387224.3367658</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>104</v>
       </c>
@@ -3064,9 +3116,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C46"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>105</v>
@@ -3075,7 +3127,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>56</v>
       </c>
@@ -3086,7 +3138,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>57</v>
       </c>
@@ -3097,7 +3149,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>58</v>
       </c>
@@ -3108,7 +3160,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>59</v>
       </c>
@@ -3119,7 +3171,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>60</v>
       </c>
@@ -3130,7 +3182,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>61</v>
       </c>
@@ -3141,7 +3193,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>62</v>
       </c>
@@ -3152,7 +3204,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>63</v>
       </c>
@@ -3163,7 +3215,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>64</v>
       </c>
@@ -3174,7 +3226,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>65</v>
       </c>
@@ -3185,7 +3237,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>66</v>
       </c>
@@ -3196,7 +3248,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>67</v>
       </c>
@@ -3207,7 +3259,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>68</v>
       </c>
@@ -3218,7 +3270,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>69</v>
       </c>
@@ -3229,7 +3281,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>70</v>
       </c>
@@ -3240,7 +3292,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>71</v>
       </c>
@@ -3251,7 +3303,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>72</v>
       </c>
@@ -3262,7 +3314,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>73</v>
       </c>
@@ -3273,7 +3325,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>74</v>
       </c>
@@ -3284,7 +3336,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>75</v>
       </c>
@@ -3295,7 +3347,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>76</v>
       </c>
@@ -3306,7 +3358,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>77</v>
       </c>
@@ -3317,7 +3369,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>78</v>
       </c>
@@ -3328,7 +3380,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>79</v>
       </c>
@@ -3339,7 +3391,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>80</v>
       </c>
@@ -3350,7 +3402,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>81</v>
       </c>
@@ -3361,7 +3413,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>82</v>
       </c>
@@ -3372,7 +3424,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>83</v>
       </c>
@@ -3383,7 +3435,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>84</v>
       </c>
@@ -3394,7 +3446,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>85</v>
       </c>
@@ -3405,7 +3457,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>86</v>
       </c>
@@ -3416,7 +3468,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>87</v>
       </c>
@@ -3427,7 +3479,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>88</v>
       </c>
@@ -3438,7 +3490,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>89</v>
       </c>
@@ -3449,7 +3501,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>90</v>
       </c>
@@ -3460,7 +3512,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>91</v>
       </c>
@@ -3471,7 +3523,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>92</v>
       </c>
@@ -3482,7 +3534,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>93</v>
       </c>
@@ -3493,7 +3545,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>94</v>
       </c>
@@ -3504,7 +3556,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>99</v>
       </c>
@@ -3515,7 +3567,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>100</v>
       </c>
@@ -3526,7 +3578,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>101</v>
       </c>
@@ -3537,7 +3589,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>102</v>
       </c>
@@ -3548,7 +3600,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>103</v>
       </c>
@@ -3559,7 +3611,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>104</v>
       </c>

</xml_diff>